<commit_message>
Fixed the duplication on archives
- makes sure that there's no duplication on the unresolved folder after the edit
</commit_message>
<xml_diff>
--- a/ViolationRecords1.xlsx
+++ b/ViolationRecords1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="133">
   <si>
     <t>NAME</t>
   </si>
@@ -413,54 +413,6 @@
   </si>
   <si>
     <t>1st Semester (S.Y. 2025-2026)</t>
-  </si>
-  <si>
-    <t>Nathan James Absel</t>
-  </si>
-  <si>
-    <t>Noisiness</t>
-  </si>
-  <si>
-    <t>Wadag, Juiliane Elize M.</t>
-  </si>
-  <si>
-    <t>BSIT 1A</t>
-  </si>
-  <si>
-    <t>Footwear</t>
-  </si>
-  <si>
-    <t>Jabinar, Jonel L.</t>
-  </si>
-  <si>
-    <t>BSIT 1E</t>
-  </si>
-  <si>
-    <t>ID still in process</t>
-  </si>
-  <si>
-    <t>Durang, Lemuel C.</t>
-  </si>
-  <si>
-    <t>Using cellphone during class</t>
-  </si>
-  <si>
-    <t>Aquino, Mark Justine</t>
-  </si>
-  <si>
-    <t>Bundalian, Angelo M.</t>
-  </si>
-  <si>
-    <t>ID late received</t>
-  </si>
-  <si>
-    <t>Pineda, Ivan Daniel</t>
-  </si>
-  <si>
-    <t>Bamuela, Francine Hope G.</t>
-  </si>
-  <si>
-    <t>Poncio, Clark Dave P.</t>
   </si>
 </sst>
 </file>
@@ -549,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -592,22 +544,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,7 +763,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="12.6640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="25.21875" customWidth="1"/>
@@ -2087,159 +2023,6 @@
       <c r="D75" s="16"/>
       <c r="E75" s="16"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="B76" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C76" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="D76" s="19">
-        <v>45937</v>
-      </c>
-      <c r="E76" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B77" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="C77" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="D77" s="19">
-        <v>45953</v>
-      </c>
-      <c r="E77" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B78" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="C78" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="D78" s="19">
-        <v>45953</v>
-      </c>
-      <c r="E78" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="B79" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C79" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="D79" s="21">
-        <v>45957</v>
-      </c>
-      <c r="E79" s="20" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="B80" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C80" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="D80" s="21">
-        <v>45958</v>
-      </c>
-      <c r="E80" s="20" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="B81" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="C81" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="D81" s="21">
-        <v>45988</v>
-      </c>
-      <c r="E81" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="B82" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="C82" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="D82" s="21">
-        <v>45988</v>
-      </c>
-      <c r="E82" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="B83" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C83" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="D83" s="22">
-        <v>45994</v>
-      </c>
-      <c r="E83" s="20" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="B84" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="C84" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="D84" s="22">
-        <v>46052</v>
-      </c>
-      <c r="E84" s="20" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Archive fix & logging logic
- duplicate record is allowed
- added delete btn per sem
 - added validation when logging an exact violation record (no duplication of date)
- fixed bug on editing sem and sy (proper saving and displaying)
</commit_message>
<xml_diff>
--- a/ViolationRecords1.xlsx
+++ b/ViolationRecords1.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B2C0CC7-116E-43B2-96C5-FC2700EC05A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="155">
   <si>
     <t>NAME</t>
   </si>
@@ -413,42 +414,108 @@
   </si>
   <si>
     <t>1st Semester (S.Y. 2025-2026)</t>
+  </si>
+  <si>
+    <t>Garcia, Jhemilyn S.</t>
+  </si>
+  <si>
+    <t>Not in Proper Uniform</t>
+  </si>
+  <si>
+    <t>Viovicente, Kevin Christian H.</t>
+  </si>
+  <si>
+    <t>Flores, Rave Benedict R.</t>
+  </si>
+  <si>
+    <t>Nadama, Clark A.</t>
+  </si>
+  <si>
+    <t>Earl John J. Gollena</t>
+  </si>
+  <si>
+    <t>Noisiness</t>
+  </si>
+  <si>
+    <t>Nathan James Absel</t>
+  </si>
+  <si>
+    <t>Wadag, Juiliane Elize M.</t>
+  </si>
+  <si>
+    <t>BSIT 1A</t>
+  </si>
+  <si>
+    <t>Footwear</t>
+  </si>
+  <si>
+    <t>Jabinar, Jonel L.</t>
+  </si>
+  <si>
+    <t>BSIT 1E</t>
+  </si>
+  <si>
+    <t>ID still in process</t>
+  </si>
+  <si>
+    <t>Durang, Lemuel C.</t>
+  </si>
+  <si>
+    <t>Using cellphone during class</t>
+  </si>
+  <si>
+    <t>Aquino, Mark Justine</t>
+  </si>
+  <si>
+    <t>Bundalian, Angelo M.</t>
+  </si>
+  <si>
+    <t>ID late received</t>
+  </si>
+  <si>
+    <t>Pineda, Ivan Daniel</t>
+  </si>
+  <si>
+    <t>Bamuela, Francine Hope G.</t>
+  </si>
+  <si>
+    <t>Poncio, Clark Dave P.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yy"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="7">
@@ -466,25 +533,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor theme="0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999816888943144"/>
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999816888943144"/>
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -501,12 +568,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -519,12 +583,6 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -539,11 +597,36 @@
     <xf numFmtId="165" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -759,20 +842,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="12.6640625" customHeight="1"/>
+  <dimension ref="A1:E89"/>
+  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.21875" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="25.25" customWidth="1"/>
+    <col min="2" max="2" width="14.75" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="5" max="5" width="33.21875" customWidth="1"/>
+    <col min="5" max="5" width="33.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -789,1232 +872,1232 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+    </row>
+    <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
         <v>45456</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>45456</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="E4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>45456</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>45456</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="E6" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>45456</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>45456</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>45456</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>45456</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>45456</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <v>45456</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="E12" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>45456</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="E13" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <v>45456</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="E14" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <v>45462</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="E15" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
         <v>45462</v>
       </c>
-      <c r="E16" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="E16" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <v>45462</v>
       </c>
-      <c r="E17" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="E17" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <v>45470</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="E18" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="4">
         <v>45509</v>
       </c>
-      <c r="E19" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="E19" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="4">
         <v>45510</v>
       </c>
-      <c r="E20" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="E20" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>45510</v>
       </c>
-      <c r="E21" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="E21" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="4">
         <v>45531</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="E23" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="E24" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="E25" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="4">
         <v>45580</v>
       </c>
-      <c r="E26" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="E26" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="4">
         <v>45580</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="E27" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="4">
         <v>45580</v>
       </c>
-      <c r="E28" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="E28" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="6">
         <v>45600</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="6">
         <v>45600</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="6">
         <v>45600</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="6">
         <v>45600</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D33" s="7">
+      <c r="D33" s="6">
         <v>45601</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="6">
         <v>45601</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
+    <row r="35" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D35" s="7">
+      <c r="D35" s="6">
         <v>45601</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
+    <row r="36" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D36" s="7">
+      <c r="D36" s="6">
         <v>45601</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
+    <row r="37" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D37" s="7">
+      <c r="D37" s="6">
         <v>45601</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D38" s="7">
+      <c r="D38" s="6">
         <v>45604</v>
       </c>
-      <c r="E38" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+      <c r="E38" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D39" s="5">
+      <c r="D39" s="4">
         <v>45611</v>
       </c>
-      <c r="E39" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
+      <c r="E39" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D40" s="5">
+      <c r="D40" s="4">
         <v>45622</v>
       </c>
-      <c r="E40" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
+      <c r="E40" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D41" s="5">
+      <c r="D41" s="4">
         <v>45622</v>
       </c>
-      <c r="E41" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
+      <c r="E41" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D42" s="5">
+      <c r="D42" s="4">
         <v>45622</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
+      <c r="E42" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D43" s="5">
+      <c r="D43" s="4">
         <v>45622</v>
       </c>
-      <c r="E43" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
+      <c r="E43" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D44" s="5">
+      <c r="D44" s="4">
         <v>45622</v>
       </c>
-      <c r="E44" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
+      <c r="E44" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D45" s="5">
+      <c r="D45" s="4">
         <v>45631</v>
       </c>
-      <c r="E45" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
+      <c r="E45" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D46" s="5">
+      <c r="D46" s="4">
         <v>45643</v>
       </c>
-      <c r="E46" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
+      <c r="E46" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D47" s="5">
+      <c r="D47" s="4">
         <v>45643</v>
       </c>
-      <c r="E47" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
+      <c r="E47" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D48" s="7">
+      <c r="D48" s="6">
         <v>45664</v>
       </c>
-      <c r="E48" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
+      <c r="E48" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D49" s="7">
+      <c r="D49" s="6">
         <v>45664</v>
       </c>
-      <c r="E49" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
+      <c r="E49" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="6">
         <v>45666</v>
       </c>
-      <c r="E50" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
+      <c r="E50" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D51" s="5">
+      <c r="D51" s="4">
         <v>45689</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="E51" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
+    <row r="52" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D52" s="5">
+      <c r="D52" s="4">
         <v>45700</v>
       </c>
-      <c r="E52" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
+      <c r="E52" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D53" s="5">
+      <c r="D53" s="4">
         <v>45714</v>
       </c>
-      <c r="E53" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
+      <c r="E53" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C54" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D54" s="5">
+      <c r="D54" s="4">
         <v>45720</v>
       </c>
-      <c r="E54" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
+      <c r="E54" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D55" s="5">
+      <c r="D55" s="4">
         <v>45721</v>
       </c>
-      <c r="E55" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" ht="13.8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="3" t="s">
+      <c r="E55" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D56" s="5">
+      <c r="D56" s="4">
         <v>45721</v>
       </c>
-      <c r="E56" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" ht="13.8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
+      <c r="E56" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-    </row>
-    <row r="58" ht="13.8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="10" t="s">
+      <c r="B57" s="14"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="14"/>
+    </row>
+    <row r="58" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="9">
         <v>45727</v>
       </c>
-      <c r="E58" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="10" t="s">
+      <c r="E58" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A59" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C59" s="11" t="s">
+      <c r="C59" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D59" s="12">
+      <c r="D59" s="9">
         <v>45728</v>
       </c>
-      <c r="E59" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="10" t="s">
+      <c r="E59" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A60" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B60" s="11" t="s">
+      <c r="B60" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="9">
         <v>45741</v>
       </c>
-      <c r="E60" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="10" t="s">
+      <c r="E60" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A61" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B61" s="11" t="s">
+      <c r="B61" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C61" s="11" t="s">
+      <c r="C61" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="9">
         <v>45741</v>
       </c>
-      <c r="E61" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="10" t="s">
+      <c r="E61" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A62" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C62" s="11" t="s">
+      <c r="C62" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="9">
         <v>45743</v>
       </c>
-      <c r="E62" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="10" t="s">
+      <c r="E62" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A63" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="11" t="s">
+      <c r="C63" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="9">
         <v>45743</v>
       </c>
-      <c r="E63" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="10" t="s">
+      <c r="E63" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A64" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B64" s="11" t="s">
+      <c r="B64" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C64" s="11" t="s">
+      <c r="C64" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="9">
         <v>45744</v>
       </c>
-      <c r="E64" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="10" t="s">
+      <c r="E64" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A65" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B65" s="11" t="s">
+      <c r="B65" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C65" s="11" t="s">
+      <c r="C65" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D65" s="12">
+      <c r="D65" s="9">
         <v>45750</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="10" t="s">
+    <row r="66" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A66" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B66" s="11" t="s">
+      <c r="B66" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D66" s="12">
+      <c r="D66" s="9">
         <v>45751</v>
       </c>
-      <c r="E66" s="13" t="s">
+      <c r="E66" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="10" t="s">
+    <row r="67" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A67" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C67" s="11" t="s">
+      <c r="C67" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="D67" s="12">
+      <c r="D67" s="9">
         <v>45770</v>
       </c>
-      <c r="E67" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="10" t="s">
+      <c r="E67" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A68" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B68" s="11" t="s">
+      <c r="B68" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C68" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D68" s="14">
+      <c r="D68" s="11">
         <v>45777</v>
       </c>
-      <c r="E68" s="13" t="s">
+      <c r="E68" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="10" t="s">
+    <row r="69" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A69" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="B69" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D69" s="12">
+      <c r="D69" s="9">
         <v>45777</v>
       </c>
-      <c r="E69" s="13" t="s">
+      <c r="E69" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="10" t="s">
+    <row r="70" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A70" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="B70" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D70" s="12">
+      <c r="D70" s="9">
         <v>45783</v>
       </c>
-      <c r="E70" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="10" t="s">
+      <c r="E70" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A71" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B71" s="11" t="s">
+      <c r="B71" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D71" s="12">
+      <c r="D71" s="9">
         <v>45783</v>
       </c>
-      <c r="E71" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="10" t="s">
+      <c r="E71" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A72" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="B72" s="11" t="s">
+      <c r="B72" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C72" s="11" t="s">
+      <c r="C72" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D72" s="12">
+      <c r="D72" s="9">
         <v>45783</v>
       </c>
-      <c r="E72" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="10" t="s">
+      <c r="E72" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A73" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B73" s="11" t="s">
+      <c r="B73" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="D73" s="12">
+      <c r="D73" s="9">
         <v>45791</v>
       </c>
-      <c r="E73" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="74" ht="13.8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="10" t="s">
+      <c r="E73" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B74" s="11" t="s">
+      <c r="B74" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D74" s="12">
+      <c r="D74" s="9">
         <v>45796</v>
       </c>
-      <c r="E74" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="75" ht="13.8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E74" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="s">
         <v>132</v>
       </c>
@@ -2022,6 +2105,244 @@
       <c r="C75" s="16"/>
       <c r="D75" s="16"/>
       <c r="E75" s="16"/>
+    </row>
+    <row r="76" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B76" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C76" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="D76" s="19">
+        <v>45903</v>
+      </c>
+      <c r="E76" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C77" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D77" s="21">
+        <v>45915</v>
+      </c>
+      <c r="E77" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B78" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C78" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D78" s="21">
+        <v>45930</v>
+      </c>
+      <c r="E78" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="B79" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C79" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D79" s="21">
+        <v>45930</v>
+      </c>
+      <c r="E79" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B80" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D80" s="19">
+        <v>45937</v>
+      </c>
+      <c r="E80" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B81" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C81" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D81" s="22">
+        <v>45937</v>
+      </c>
+      <c r="E81" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B82" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="C82" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D82" s="22">
+        <v>45953</v>
+      </c>
+      <c r="E82" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="B83" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C83" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D83" s="22">
+        <v>45953</v>
+      </c>
+      <c r="E83" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="B84" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C84" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D84" s="19">
+        <v>45957</v>
+      </c>
+      <c r="E84" s="20" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B85" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C85" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D85" s="19">
+        <v>45958</v>
+      </c>
+      <c r="E85" s="20" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="B86" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C86" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="D86" s="19">
+        <v>45988</v>
+      </c>
+      <c r="E86" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="D87" s="19">
+        <v>45988</v>
+      </c>
+      <c r="E87" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B88" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C88" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D88" s="21">
+        <v>45994</v>
+      </c>
+      <c r="E88" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="B89" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D89" s="21">
+        <v>46052</v>
+      </c>
+      <c r="E89" s="20" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>